<commit_message>
Sync Stage_Storage with local survey edits (sans Ø900)
Match user WSE/area table (36.01, 37.28@2198, 37.40, 40.00) so rebuilds
no longer overwrite the local Stage_Storage values.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
@@ -946,12 +946,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Compose_1200'!$A$13:$A$59</f>
+              <f>'Compose_1200'!$A$13:$A$64</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Compose_1200'!$J$13:$J$59</f>
+              <f>'Compose_1200'!$J$13:$J$64</f>
             </numRef>
           </val>
         </ser>
@@ -978,12 +978,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Compose_1200'!$A$13:$A$59</f>
+              <f>'Compose_1200'!$A$13:$A$64</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Compose_1200'!$H$13:$H$59</f>
+              <f>'Compose_1200'!$H$13:$H$64</f>
             </numRef>
           </val>
         </ser>
@@ -1010,12 +1010,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'Compose_1200'!$A$13:$A$59</f>
+              <f>'Compose_1200'!$A$13:$A$64</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Compose_1200'!$I$13:$I$59</f>
+              <f>'Compose_1200'!$I$13:$I$64</f>
             </numRef>
           </val>
         </ser>
@@ -2028,7 +2028,7 @@
         </is>
       </c>
       <c r="B38" s="14">
-        <f>IF(B36&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B36&gt;=Stage_Storage!E18,"Hors table — etendre leve",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1))+(B36-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))))</f>
+        <f>IF(B36&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B36&gt;=Stage_Storage!E18,"Hors table (&gt;=40.0 m — etendre leve)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1))+(B36-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B36,Stage_Storage!$E$11:$E$18,1)))))</f>
         <v/>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
         </is>
       </c>
       <c r="B44" s="14">
-        <f>IF(B42&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B42&gt;=Stage_Storage!E18,"Hors table — etendre leve",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1))+(B42-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)))))</f>
+        <f>IF(B42&lt;=Stage_Storage!E11,Stage_Storage!A11,IF(B42&gt;=Stage_Storage!E18,"Hors table (&gt;=40.0 m — etendre leve)",INDEX(Stage_Storage!$A$11:$A$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1))+(B42-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)))/(INDEX(Stage_Storage!$E$11:$E$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)))*(INDEX(Stage_Storage!$A$11:$A$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(B42,Stage_Storage!$E$11:$E$18,1)))))</f>
         <v/>
       </c>
     </row>
@@ -4942,7 +4942,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>V_pas = 0.5*(A_bas+A_haut)*dWSE. Remplacez les aires par votre nouveau leve (plus d'aire attendue sans emprise Ø900). 37.28 m = ancienne limite patron.</t>
+          <t>V_pas = 0.5*(A_bas+A_haut)*dWSE. Remplacez les aires par votre nouveau leve (plus d'aire attendue sans emprise Ø900). Surfaces jaunes synchronisees avec votre copie locale (sept. 2026). 37.28 m = cote cle / limite patron.</t>
         </is>
       </c>
     </row>
@@ -5028,10 +5028,10 @@
     </row>
     <row r="13">
       <c r="A13" s="28" t="n">
-        <v>36</v>
+        <v>36.01</v>
       </c>
       <c r="B13" s="10" t="n">
-        <v>280</v>
+        <v>419</v>
       </c>
       <c r="C13" s="28">
         <f>A13-A12</f>
@@ -5106,7 +5106,7 @@
         <v>37.28</v>
       </c>
       <c r="B16" s="10" t="n">
-        <v>850</v>
+        <v>2198</v>
       </c>
       <c r="C16" s="31">
         <f>A16-A15</f>
@@ -5122,16 +5122,16 @@
       </c>
       <c r="F16" s="33" t="inlineStr">
         <is>
-          <t>Limite patron (ex) — a recalibrer</t>
+          <t>Limite patron / cote cle</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="28" t="n">
-        <v>37.5</v>
+        <v>37.4</v>
       </c>
       <c r="B17" s="10" t="n">
-        <v>1100</v>
+        <v>1516</v>
       </c>
       <c r="C17" s="28">
         <f>A17-A16</f>
@@ -5153,10 +5153,10 @@
     </row>
     <row r="18">
       <c r="A18" s="28" t="n">
-        <v>39.5</v>
+        <v>40</v>
       </c>
       <c r="B18" s="10" t="n">
-        <v>2800</v>
+        <v>3746</v>
       </c>
       <c r="C18" s="28">
         <f>A18-A17</f>
@@ -5232,7 +5232,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K59"/>
+  <dimension ref="A1:K64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7302,6 +7302,211 @@
       </c>
       <c r="J59" s="9">
         <f>H59+I59</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="28" t="n">
+        <v>39.58</v>
+      </c>
+      <c r="B60" s="28">
+        <f>A60-$B$10</f>
+        <v/>
+      </c>
+      <c r="C60" s="28">
+        <f>MAX(0,A60-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D60" s="19">
+        <f>IF(C60&lt;=0,0,($B$5+$B$7*C60)*C60)</f>
+        <v/>
+      </c>
+      <c r="E60" s="18">
+        <f>D60*$B$9</f>
+        <v/>
+      </c>
+      <c r="F60" s="18">
+        <f>IF(A60&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A60&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1))+(A60-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A60,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G60" s="24">
+        <f>E60+F60</f>
+        <v/>
+      </c>
+      <c r="H60" s="19">
+        <f>IF(B60&lt;=0,0,IF(B60&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1))+(B60-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B60,Courbe_QH_1200!$A$20:$A$80,1)))))</f>
+        <v/>
+      </c>
+      <c r="I60" s="19">
+        <f>IF(C60&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D60*IF(($B$5+2*C60*SQRT(1+$B$7^2))&lt;=0,0,((D60/($B$5+2*C60*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J60" s="9">
+        <f>H60+I60</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="28" t="n">
+        <v>39.68</v>
+      </c>
+      <c r="B61" s="28">
+        <f>A61-$B$10</f>
+        <v/>
+      </c>
+      <c r="C61" s="28">
+        <f>MAX(0,A61-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D61" s="19">
+        <f>IF(C61&lt;=0,0,($B$5+$B$7*C61)*C61)</f>
+        <v/>
+      </c>
+      <c r="E61" s="18">
+        <f>D61*$B$9</f>
+        <v/>
+      </c>
+      <c r="F61" s="18">
+        <f>IF(A61&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A61&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1))+(A61-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A61,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G61" s="24">
+        <f>E61+F61</f>
+        <v/>
+      </c>
+      <c r="H61" s="19">
+        <f>IF(B61&lt;=0,0,IF(B61&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1))+(B61-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B61,Courbe_QH_1200!$A$20:$A$80,1)))))</f>
+        <v/>
+      </c>
+      <c r="I61" s="19">
+        <f>IF(C61&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D61*IF(($B$5+2*C61*SQRT(1+$B$7^2))&lt;=0,0,((D61/($B$5+2*C61*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J61" s="9">
+        <f>H61+I61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="28" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="B62" s="28">
+        <f>A62-$B$10</f>
+        <v/>
+      </c>
+      <c r="C62" s="28">
+        <f>MAX(0,A62-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D62" s="19">
+        <f>IF(C62&lt;=0,0,($B$5+$B$7*C62)*C62)</f>
+        <v/>
+      </c>
+      <c r="E62" s="18">
+        <f>D62*$B$9</f>
+        <v/>
+      </c>
+      <c r="F62" s="18">
+        <f>IF(A62&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A62&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1))+(A62-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A62,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G62" s="24">
+        <f>E62+F62</f>
+        <v/>
+      </c>
+      <c r="H62" s="19">
+        <f>IF(B62&lt;=0,0,IF(B62&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1))+(B62-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B62,Courbe_QH_1200!$A$20:$A$80,1)))))</f>
+        <v/>
+      </c>
+      <c r="I62" s="19">
+        <f>IF(C62&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D62*IF(($B$5+2*C62*SQRT(1+$B$7^2))&lt;=0,0,((D62/($B$5+2*C62*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J62" s="9">
+        <f>H62+I62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="28" t="n">
+        <v>39.88</v>
+      </c>
+      <c r="B63" s="28">
+        <f>A63-$B$10</f>
+        <v/>
+      </c>
+      <c r="C63" s="28">
+        <f>MAX(0,A63-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D63" s="19">
+        <f>IF(C63&lt;=0,0,($B$5+$B$7*C63)*C63)</f>
+        <v/>
+      </c>
+      <c r="E63" s="18">
+        <f>D63*$B$9</f>
+        <v/>
+      </c>
+      <c r="F63" s="18">
+        <f>IF(A63&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A63&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1))+(A63-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A63,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G63" s="24">
+        <f>E63+F63</f>
+        <v/>
+      </c>
+      <c r="H63" s="19">
+        <f>IF(B63&lt;=0,0,IF(B63&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1))+(B63-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B63,Courbe_QH_1200!$A$20:$A$80,1)))))</f>
+        <v/>
+      </c>
+      <c r="I63" s="19">
+        <f>IF(C63&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D63*IF(($B$5+2*C63*SQRT(1+$B$7^2))&lt;=0,0,((D63/($B$5+2*C63*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J63" s="9">
+        <f>H63+I63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="28" t="n">
+        <v>39.98</v>
+      </c>
+      <c r="B64" s="28">
+        <f>A64-$B$10</f>
+        <v/>
+      </c>
+      <c r="C64" s="28">
+        <f>MAX(0,A64-$B$4)</f>
+        <v/>
+      </c>
+      <c r="D64" s="19">
+        <f>IF(C64&lt;=0,0,($B$5+$B$7*C64)*C64)</f>
+        <v/>
+      </c>
+      <c r="E64" s="18">
+        <f>D64*$B$9</f>
+        <v/>
+      </c>
+      <c r="F64" s="18">
+        <f>IF(A64&lt;=INDEX(Stage_Storage!$A$11:$A$18,1),INDEX(Stage_Storage!$E$11:$E$18,1),IF(A64&gt;=INDEX(Stage_Storage!$A$11:$A$18,ROWS(Stage_Storage!$A$11:$A$18)),INDEX(Stage_Storage!$E$11:$E$18,ROWS(Stage_Storage!$E$11:$E$18)),INDEX(Stage_Storage!$E$11:$E$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1))+(A64-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)))/(INDEX(Stage_Storage!$A$11:$A$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$A$11:$A$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)))*(INDEX(Stage_Storage!$E$11:$E$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)+1)-INDEX(Stage_Storage!$E$11:$E$18,MATCH(A64,Stage_Storage!$A$11:$A$18,1)))))</f>
+        <v/>
+      </c>
+      <c r="G64" s="24">
+        <f>E64+F64</f>
+        <v/>
+      </c>
+      <c r="H64" s="19">
+        <f>IF(B64&lt;=0,0,IF(B64&gt;=INDEX(Courbe_QH_1200!$A$20:$A$80,ROWS(Courbe_QH_1200!$A$20:$A$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,ROWS(Courbe_QH_1200!$E$20:$E$80)),INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1))+(B64-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))/(INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$A$20:$A$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))*(INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)+1)-INDEX(Courbe_QH_1200!$E$20:$E$80,MATCH(B64,Courbe_QH_1200!$A$20:$A$80,1)))))</f>
+        <v/>
+      </c>
+      <c r="I64" s="19">
+        <f>IF(C64&lt;=0,0,IF($B$6&lt;=0,0,(1/$B$6)*D64*IF(($B$5+2*C64*SQRT(1+$B$7^2))&lt;=0,0,((D64/($B$5+2*C64*SQRT(1+$B$7^2)))^(2/3)))*SQRT($B$8)))</f>
+        <v/>
+      </c>
+      <c r="J64" s="9">
+        <f>H64+I64</f>
         <v/>
       </c>
     </row>
@@ -7457,11 +7662,11 @@
         <v/>
       </c>
       <c r="C11" s="19">
-        <f>IF(F10&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F10&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F10,Compose_1200!$G$13:$G$59,1))+(F10-INDEX(Compose_1200!$G$13:$G$59,MATCH(F10,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F10,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F10,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F10,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F10,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F10&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F10&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F10,Compose_1200!$G$13:$G$64,1))+(F10-INDEX(Compose_1200!$G$13:$G$64,MATCH(F10,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F10,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F10,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F10,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F10,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D11" s="19">
-        <f>IF(F10&lt;=0.01,MIN(0.5*(B10+B11),$B$4),IF(C11&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C11&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C11,Compose_1200!$A$13:$A$59,1))+(C11-INDEX(Compose_1200!$A$13:$A$59,MATCH(C11,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C11,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C11,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C11,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C11,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F10&lt;=0.01,MIN(0.5*(B10+B11),$B$4),IF(C11&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C11&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C11,Compose_1200!$A$13:$A$64,1))+(C11-INDEX(Compose_1200!$A$13:$A$64,MATCH(C11,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C11,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C11,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C11,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C11,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E11" s="18">
@@ -7487,11 +7692,11 @@
         <v/>
       </c>
       <c r="C12" s="19">
-        <f>IF(F11&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F11&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F11,Compose_1200!$G$13:$G$59,1))+(F11-INDEX(Compose_1200!$G$13:$G$59,MATCH(F11,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F11,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F11,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F11,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F11,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F11&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F11&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F11,Compose_1200!$G$13:$G$64,1))+(F11-INDEX(Compose_1200!$G$13:$G$64,MATCH(F11,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F11,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F11,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F11,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F11,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D12" s="19">
-        <f>IF(F11&lt;=0.01,MIN(0.5*(B11+B12),$B$4),IF(C12&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C12&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C12,Compose_1200!$A$13:$A$59,1))+(C12-INDEX(Compose_1200!$A$13:$A$59,MATCH(C12,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C12,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C12,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C12,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C12,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F11&lt;=0.01,MIN(0.5*(B11+B12),$B$4),IF(C12&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C12&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C12,Compose_1200!$A$13:$A$64,1))+(C12-INDEX(Compose_1200!$A$13:$A$64,MATCH(C12,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C12,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C12,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C12,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C12,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E12" s="18">
@@ -7517,11 +7722,11 @@
         <v/>
       </c>
       <c r="C13" s="19">
-        <f>IF(F12&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F12&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F12,Compose_1200!$G$13:$G$59,1))+(F12-INDEX(Compose_1200!$G$13:$G$59,MATCH(F12,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F12,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F12,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F12,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F12,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F12&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F12&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F12,Compose_1200!$G$13:$G$64,1))+(F12-INDEX(Compose_1200!$G$13:$G$64,MATCH(F12,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F12,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F12,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F12,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F12,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D13" s="19">
-        <f>IF(F12&lt;=0.01,MIN(0.5*(B12+B13),$B$4),IF(C13&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C13&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C13,Compose_1200!$A$13:$A$59,1))+(C13-INDEX(Compose_1200!$A$13:$A$59,MATCH(C13,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C13,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C13,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C13,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C13,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F12&lt;=0.01,MIN(0.5*(B12+B13),$B$4),IF(C13&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C13&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C13,Compose_1200!$A$13:$A$64,1))+(C13-INDEX(Compose_1200!$A$13:$A$64,MATCH(C13,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C13,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C13,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C13,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C13,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E13" s="18">
@@ -7547,11 +7752,11 @@
         <v/>
       </c>
       <c r="C14" s="19">
-        <f>IF(F13&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F13&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F13,Compose_1200!$G$13:$G$59,1))+(F13-INDEX(Compose_1200!$G$13:$G$59,MATCH(F13,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F13,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F13,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F13,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F13,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F13&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F13&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F13,Compose_1200!$G$13:$G$64,1))+(F13-INDEX(Compose_1200!$G$13:$G$64,MATCH(F13,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F13,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F13,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F13,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F13,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D14" s="19">
-        <f>IF(F13&lt;=0.01,MIN(0.5*(B13+B14),$B$4),IF(C14&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C14&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C14,Compose_1200!$A$13:$A$59,1))+(C14-INDEX(Compose_1200!$A$13:$A$59,MATCH(C14,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C14,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C14,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C14,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C14,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F13&lt;=0.01,MIN(0.5*(B13+B14),$B$4),IF(C14&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C14&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C14,Compose_1200!$A$13:$A$64,1))+(C14-INDEX(Compose_1200!$A$13:$A$64,MATCH(C14,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C14,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C14,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C14,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C14,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E14" s="18">
@@ -7577,11 +7782,11 @@
         <v/>
       </c>
       <c r="C15" s="19">
-        <f>IF(F14&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F14&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F14,Compose_1200!$G$13:$G$59,1))+(F14-INDEX(Compose_1200!$G$13:$G$59,MATCH(F14,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F14,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F14,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F14,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F14,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F14&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F14&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F14,Compose_1200!$G$13:$G$64,1))+(F14-INDEX(Compose_1200!$G$13:$G$64,MATCH(F14,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F14,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F14,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F14,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F14,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D15" s="19">
-        <f>IF(F14&lt;=0.01,MIN(0.5*(B14+B15),$B$4),IF(C15&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C15&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C15,Compose_1200!$A$13:$A$59,1))+(C15-INDEX(Compose_1200!$A$13:$A$59,MATCH(C15,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C15,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C15,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C15,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C15,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F14&lt;=0.01,MIN(0.5*(B14+B15),$B$4),IF(C15&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C15&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C15,Compose_1200!$A$13:$A$64,1))+(C15-INDEX(Compose_1200!$A$13:$A$64,MATCH(C15,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C15,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C15,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C15,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C15,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E15" s="18">
@@ -7607,11 +7812,11 @@
         <v/>
       </c>
       <c r="C16" s="19">
-        <f>IF(F15&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F15&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F15,Compose_1200!$G$13:$G$59,1))+(F15-INDEX(Compose_1200!$G$13:$G$59,MATCH(F15,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F15,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F15,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F15,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F15,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F15&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F15&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F15,Compose_1200!$G$13:$G$64,1))+(F15-INDEX(Compose_1200!$G$13:$G$64,MATCH(F15,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F15,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F15,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F15,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F15,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D16" s="19">
-        <f>IF(F15&lt;=0.01,MIN(0.5*(B15+B16),$B$4),IF(C16&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C16&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C16,Compose_1200!$A$13:$A$59,1))+(C16-INDEX(Compose_1200!$A$13:$A$59,MATCH(C16,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C16,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C16,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C16,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C16,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F15&lt;=0.01,MIN(0.5*(B15+B16),$B$4),IF(C16&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C16&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C16,Compose_1200!$A$13:$A$64,1))+(C16-INDEX(Compose_1200!$A$13:$A$64,MATCH(C16,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C16,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C16,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C16,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C16,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E16" s="18">
@@ -7637,11 +7842,11 @@
         <v/>
       </c>
       <c r="C17" s="19">
-        <f>IF(F16&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F16&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F16,Compose_1200!$G$13:$G$59,1))+(F16-INDEX(Compose_1200!$G$13:$G$59,MATCH(F16,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F16,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F16,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F16,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F16,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F16&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F16&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F16,Compose_1200!$G$13:$G$64,1))+(F16-INDEX(Compose_1200!$G$13:$G$64,MATCH(F16,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F16,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F16,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F16,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F16,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D17" s="19">
-        <f>IF(F16&lt;=0.01,MIN(0.5*(B16+B17),$B$4),IF(C17&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C17&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C17,Compose_1200!$A$13:$A$59,1))+(C17-INDEX(Compose_1200!$A$13:$A$59,MATCH(C17,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C17,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C17,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C17,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C17,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F16&lt;=0.01,MIN(0.5*(B16+B17),$B$4),IF(C17&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C17&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C17,Compose_1200!$A$13:$A$64,1))+(C17-INDEX(Compose_1200!$A$13:$A$64,MATCH(C17,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C17,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C17,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C17,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C17,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E17" s="18">
@@ -7667,11 +7872,11 @@
         <v/>
       </c>
       <c r="C18" s="19">
-        <f>IF(F17&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F17&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F17,Compose_1200!$G$13:$G$59,1))+(F17-INDEX(Compose_1200!$G$13:$G$59,MATCH(F17,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F17,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F17,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F17,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F17,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F17&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F17&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F17,Compose_1200!$G$13:$G$64,1))+(F17-INDEX(Compose_1200!$G$13:$G$64,MATCH(F17,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F17,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F17,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F17,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F17,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D18" s="19">
-        <f>IF(F17&lt;=0.01,MIN(0.5*(B17+B18),$B$4),IF(C18&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C18&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C18,Compose_1200!$A$13:$A$59,1))+(C18-INDEX(Compose_1200!$A$13:$A$59,MATCH(C18,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C18,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C18,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C18,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C18,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F17&lt;=0.01,MIN(0.5*(B17+B18),$B$4),IF(C18&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C18&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C18,Compose_1200!$A$13:$A$64,1))+(C18-INDEX(Compose_1200!$A$13:$A$64,MATCH(C18,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C18,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C18,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C18,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C18,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E18" s="18">
@@ -7697,11 +7902,11 @@
         <v/>
       </c>
       <c r="C19" s="19">
-        <f>IF(F18&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F18&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F18,Compose_1200!$G$13:$G$59,1))+(F18-INDEX(Compose_1200!$G$13:$G$59,MATCH(F18,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F18,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F18,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F18,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F18,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F18&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F18&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F18,Compose_1200!$G$13:$G$64,1))+(F18-INDEX(Compose_1200!$G$13:$G$64,MATCH(F18,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F18,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F18,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F18,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F18,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D19" s="19">
-        <f>IF(F18&lt;=0.01,MIN(0.5*(B18+B19),$B$4),IF(C19&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C19&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C19,Compose_1200!$A$13:$A$59,1))+(C19-INDEX(Compose_1200!$A$13:$A$59,MATCH(C19,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C19,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C19,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C19,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C19,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F18&lt;=0.01,MIN(0.5*(B18+B19),$B$4),IF(C19&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C19&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C19,Compose_1200!$A$13:$A$64,1))+(C19-INDEX(Compose_1200!$A$13:$A$64,MATCH(C19,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C19,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C19,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C19,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C19,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E19" s="18">
@@ -7727,11 +7932,11 @@
         <v/>
       </c>
       <c r="C20" s="19">
-        <f>IF(F19&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F19&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F19,Compose_1200!$G$13:$G$59,1))+(F19-INDEX(Compose_1200!$G$13:$G$59,MATCH(F19,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F19,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F19,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F19,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F19,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F19&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F19&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F19,Compose_1200!$G$13:$G$64,1))+(F19-INDEX(Compose_1200!$G$13:$G$64,MATCH(F19,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F19,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F19,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F19,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F19,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D20" s="19">
-        <f>IF(F19&lt;=0.01,MIN(0.5*(B19+B20),$B$4),IF(C20&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C20&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C20,Compose_1200!$A$13:$A$59,1))+(C20-INDEX(Compose_1200!$A$13:$A$59,MATCH(C20,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C20,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C20,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C20,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C20,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F19&lt;=0.01,MIN(0.5*(B19+B20),$B$4),IF(C20&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C20&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C20,Compose_1200!$A$13:$A$64,1))+(C20-INDEX(Compose_1200!$A$13:$A$64,MATCH(C20,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C20,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C20,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C20,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C20,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E20" s="18">
@@ -7757,11 +7962,11 @@
         <v/>
       </c>
       <c r="C21" s="19">
-        <f>IF(F20&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F20&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F20,Compose_1200!$G$13:$G$59,1))+(F20-INDEX(Compose_1200!$G$13:$G$59,MATCH(F20,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F20,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F20,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F20,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F20,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F20&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F20&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F20,Compose_1200!$G$13:$G$64,1))+(F20-INDEX(Compose_1200!$G$13:$G$64,MATCH(F20,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F20,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F20,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F20,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F20,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D21" s="19">
-        <f>IF(F20&lt;=0.01,MIN(0.5*(B20+B21),$B$4),IF(C21&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C21&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C21,Compose_1200!$A$13:$A$59,1))+(C21-INDEX(Compose_1200!$A$13:$A$59,MATCH(C21,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C21,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C21,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C21,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C21,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F20&lt;=0.01,MIN(0.5*(B20+B21),$B$4),IF(C21&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C21&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C21,Compose_1200!$A$13:$A$64,1))+(C21-INDEX(Compose_1200!$A$13:$A$64,MATCH(C21,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C21,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C21,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C21,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C21,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E21" s="18">
@@ -7787,11 +7992,11 @@
         <v/>
       </c>
       <c r="C22" s="19">
-        <f>IF(F21&lt;=INDEX(Compose_1200!$G$13:$G$59,1),INDEX(Compose_1200!$A$13:$A$59,1),IF(F21&gt;=INDEX(Compose_1200!$G$13:$G$59,ROWS(Compose_1200!$G$13:$G$59)),INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$A$13:$A$59,MATCH(F21,Compose_1200!$G$13:$G$59,1))+(F21-INDEX(Compose_1200!$G$13:$G$59,MATCH(F21,Compose_1200!$G$13:$G$59,1)))/(INDEX(Compose_1200!$G$13:$G$59,MATCH(F21,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$G$13:$G$59,MATCH(F21,Compose_1200!$G$13:$G$59,1)))*(INDEX(Compose_1200!$A$13:$A$59,MATCH(F21,Compose_1200!$G$13:$G$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(F21,Compose_1200!$G$13:$G$59,1)))))</f>
+        <f>IF(F21&lt;=INDEX(Compose_1200!$G$13:$G$64,1),INDEX(Compose_1200!$A$13:$A$64,1),IF(F21&gt;=INDEX(Compose_1200!$G$13:$G$64,ROWS(Compose_1200!$G$13:$G$64)),INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$A$13:$A$64,MATCH(F21,Compose_1200!$G$13:$G$64,1))+(F21-INDEX(Compose_1200!$G$13:$G$64,MATCH(F21,Compose_1200!$G$13:$G$64,1)))/(INDEX(Compose_1200!$G$13:$G$64,MATCH(F21,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$G$13:$G$64,MATCH(F21,Compose_1200!$G$13:$G$64,1)))*(INDEX(Compose_1200!$A$13:$A$64,MATCH(F21,Compose_1200!$G$13:$G$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(F21,Compose_1200!$G$13:$G$64,1)))))</f>
         <v/>
       </c>
       <c r="D22" s="19">
-        <f>IF(F21&lt;=0.01,MIN(0.5*(B21+B22),$B$4),IF(C22&lt;=INDEX(Compose_1200!$A$13:$A$59,1),INDEX(Compose_1200!$J$13:$J$59,1),IF(C22&gt;=INDEX(Compose_1200!$A$13:$A$59,ROWS(Compose_1200!$A$13:$A$59)),INDEX(Compose_1200!$J$13:$J$59,ROWS(Compose_1200!$J$13:$J$59)),INDEX(Compose_1200!$J$13:$J$59,MATCH(C22,Compose_1200!$A$13:$A$59,1))+(C22-INDEX(Compose_1200!$A$13:$A$59,MATCH(C22,Compose_1200!$A$13:$A$59,1)))/(INDEX(Compose_1200!$A$13:$A$59,MATCH(C22,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$A$13:$A$59,MATCH(C22,Compose_1200!$A$13:$A$59,1)))*(INDEX(Compose_1200!$J$13:$J$59,MATCH(C22,Compose_1200!$A$13:$A$59,1)+1)-INDEX(Compose_1200!$J$13:$J$59,MATCH(C22,Compose_1200!$A$13:$A$59,1))))))</f>
+        <f>IF(F21&lt;=0.01,MIN(0.5*(B21+B22),$B$4),IF(C22&lt;=INDEX(Compose_1200!$A$13:$A$64,1),INDEX(Compose_1200!$J$13:$J$64,1),IF(C22&gt;=INDEX(Compose_1200!$A$13:$A$64,ROWS(Compose_1200!$A$13:$A$64)),INDEX(Compose_1200!$J$13:$J$64,ROWS(Compose_1200!$J$13:$J$64)),INDEX(Compose_1200!$J$13:$J$64,MATCH(C22,Compose_1200!$A$13:$A$64,1))+(C22-INDEX(Compose_1200!$A$13:$A$64,MATCH(C22,Compose_1200!$A$13:$A$64,1)))/(INDEX(Compose_1200!$A$13:$A$64,MATCH(C22,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$A$13:$A$64,MATCH(C22,Compose_1200!$A$13:$A$64,1)))*(INDEX(Compose_1200!$J$13:$J$64,MATCH(C22,Compose_1200!$A$13:$A$64,1)+1)-INDEX(Compose_1200!$J$13:$J$64,MATCH(C22,Compose_1200!$A$13:$A$64,1))))))</f>
         <v/>
       </c>
       <c r="E22" s="18">

</xml_diff>

<commit_message>
Force blank Role at WSE 37.28 and remove leftover label text
Ensure Stage_Storage F16 stays empty and help text no longer says
limite patron, so local refresh cannot resurrect that Role label.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
@@ -4942,7 +4942,7 @@
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>V_pas = 0.5*(A_bas+A_haut)*dWSE. Remplacez les aires par votre nouveau leve (plus d'aire attendue sans emprise Ø900). Surfaces jaunes synchronisees avec votre copie locale (sept. 2026). 37.28 m = cote cle / limite patron.</t>
+          <t>V_pas = 0.5*(A_bas+A_haut)*dWSE. Remplacez les aires par votre nouveau leve (plus d'aire attendue sans emprise Ø900). Surfaces jaunes synchronisees avec votre copie locale. Ligne 37.28 m: Role laisse vide (comme votre fichier local).</t>
         </is>
       </c>
     </row>
@@ -5120,11 +5120,7 @@
         <f>E15+D16</f>
         <v/>
       </c>
-      <c r="F16" s="33" t="inlineStr">
-        <is>
-          <t>Limite patron / cote cle</t>
-        </is>
-      </c>
+      <c r="F16" s="33" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="28" t="n">

</xml_diff>

<commit_message>
Update Sans_900: combined Z1+Z2 survey, crest 37.40, V_ditch switch
Align the no-Ø900 workbook with latest site assumptions: one pond from
Zone1+Zone2 areas, city WSE limit 37.40 m, and B25=0 survey-only storage.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
@@ -1682,7 +1682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -1703,7 +1703,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hypotheses: le Ø900 est elimine; plus d'aire de retention. Entree = hydrogramme (Ø1500). Sortie = Ø1200. Option: fossé/berme au-dessus d'une cote crest. Cellules JAUNES = entrees.</t>
+          <t>Hypotheses: le Ø900 est elimine; un seul bassin (surfaces = Zone1+Zone2 du leve). Entree = hydrogramme (Ø1500). Sortie = Ø1200. Limite ville WSE = 37.40 m (B27). B25=0 → volume = leve seul (pas de V_ditch). Cellules JAUNES = entrees. Aluminium ondule: augmenter n (ex. 0.024) sur Courbe_QH_1200.</t>
         </is>
       </c>
     </row>
@@ -1745,6 +1745,11 @@
       <c r="B10" s="5" t="n">
         <v>0.013</v>
       </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>beton ~0.013; aluminium ondule typ. 0.022–0.025 (changer aussi Courbe_QH_1200)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1890,11 +1895,26 @@
         </is>
       </c>
       <c r="B24" s="10" t="n">
-        <v>4000</v>
+        <v>2320</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Plus grande qu'avant (plus d'aire retention) — affiner avec le leve</t>
+          <t>Raccourci Methode B seulement (H=V/A). Ex. A@37.40≈2320 — PAS un 2e bassin</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Inclure V_ditch trapeze? (1=oui, 0=leve seul)</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0 = recommande si Stage_Storage contient deja le fosse (V=leve seul; Q_overflow garde b,z,L). 1 = ajoute V_ditch = A_trapeze x L (risque double volume).</t>
         </is>
       </c>
     </row>
@@ -1912,11 +1932,11 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>37.28</v>
+        <v>37.4</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Si WSE &lt; crest → Q_overflow = 0</t>
+          <t>Limite ville = 37.40 m par defaut. Si WSE &lt; crest → Q_overflow = 0</t>
         </is>
       </c>
     </row>
@@ -1986,10 +2006,9 @@
           <t>Q_1200(WSE) + Q_overflow(WSE)</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>V = V_pond + V_ditch — Compose_1200 + Calcul_C</t>
-        </is>
+      <c r="C33">
+        <f>IF(B25=1,"V=V_pond+V_ditch","V=V_pond (leve seul, B25=0)") — Compose_1200 + Calcul_C</f>
+        <v/>
       </c>
     </row>
     <row r="35">
@@ -2097,14 +2116,14 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>Resultats Methode C — Ø1200 + overflow (Calcul_C)</t>
+          <t>Resultats Methode C — Ø1200 + Q_overflow (V via B25)</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vmax_C (m3) = max(V_pond+V_ditch)</t>
+          <t>Vmax_C (m3) = max(V_total)</t>
         </is>
       </c>
       <c r="B48" s="13">
@@ -2167,29 +2186,37 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>• Plus d'aire de bassin: augmenter les surfaces jaunes sur Stage_Storage (et/ou Aire B24).</t>
+          <t>• Stage_Storage = Z1+Z2 (sans Ø900). Editer jaune; limite ville 37.40 m (B27 / ligne orange).</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>• Methode A: 1re estimation. B: rating FHWA pipe. C: pipe + fosse si WSE depasse le crest.</t>
+          <t>• B25=0: V Methode C = leve seul. B25=1: +V_ditch trapeze. Q_overflow toujours actif si WSE&gt;crest.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>• Verifier la capacite/vitesse aval avec Qout(t) de Calcul_B ou C (pointe plus haute qu'avec Ø900).</t>
+          <t>• Methode A: 1re estimation. B: FHWA pipe (Aire B24). C: pipe + Q_overflow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>• Verifier pointe aval (Ø1200 livre plus que l'ancien Ø900).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A2:F3"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A58:F58"/>
     <mergeCell ref="A56:F56"/>
     <mergeCell ref="A55:F55"/>
     <mergeCell ref="A57:F57"/>
@@ -4921,7 +4948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -4935,14 +4962,14 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Stage–storage du leve (bassin AGRANDI sans Ø900) — editer surfaces jaunes</t>
+          <t>Stage–storage COMBINE (Zone1+Zone2) — bassin SANS Ø900 — editer jaune</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="30" t="inlineStr">
         <is>
-          <t>V_pas = 0.5*(A_bas+A_haut)*dWSE. Remplacez les aires par votre nouveau leve (plus d'aire attendue sans emprise Ø900). Surfaces jaunes synchronisees avec votre copie locale. Ligne 37.28 m: Role laisse vide (comme votre fichier local).</t>
+          <t>V_pas = 0.5*(A_bas+A_haut)*dWSE. Aires = somme Z1+Z2 du leve deux zones (scenario sans ponceau Ø900 intermediaire). Jaune = WSE et Surface editables (AutoCAD). Orange = 37.40 m limite ville. Ancien seuil etude 37.28 reste dans la table.</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5033,7 @@
         <v>35.5</v>
       </c>
       <c r="B12" s="10" t="n">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C12" s="28">
         <f>A12-A11</f>
@@ -5022,7 +5049,7 @@
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer</t>
+          <t>Levé Z1+Z2 — éditer si AutoCAD diffère</t>
         </is>
       </c>
     </row>
@@ -5031,7 +5058,7 @@
         <v>36.01</v>
       </c>
       <c r="B13" s="10" t="n">
-        <v>419</v>
+        <v>429</v>
       </c>
       <c r="C13" s="28">
         <f>A13-A12</f>
@@ -5047,7 +5074,7 @@
       </c>
       <c r="F13" s="26" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer</t>
+          <t>Levé Z1+Z2</t>
         </is>
       </c>
     </row>
@@ -5056,7 +5083,7 @@
         <v>36.5</v>
       </c>
       <c r="B14" s="10" t="n">
-        <v>480</v>
+        <v>530</v>
       </c>
       <c r="C14" s="28">
         <f>A14-A13</f>
@@ -5072,7 +5099,7 @@
       </c>
       <c r="F14" s="26" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer</t>
+          <t>Levé Z1+Z2</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5108,7 @@
         <v>37</v>
       </c>
       <c r="B15" s="10" t="n">
-        <v>720</v>
+        <v>740</v>
       </c>
       <c r="C15" s="28">
         <f>A15-A14</f>
@@ -5097,7 +5124,7 @@
       </c>
       <c r="F15" s="26" t="inlineStr">
         <is>
-          <t>Placeholder — remplacer</t>
+          <t>Levé Z1+Z2</t>
         </is>
       </c>
     </row>
@@ -5106,7 +5133,7 @@
         <v>37.28</v>
       </c>
       <c r="B16" s="10" t="n">
-        <v>2198</v>
+        <v>2200</v>
       </c>
       <c r="C16" s="31">
         <f>A16-A15</f>
@@ -5120,30 +5147,34 @@
         <f>E15+D16</f>
         <v/>
       </c>
-      <c r="F16" s="33" t="n"/>
+      <c r="F16" s="33" t="inlineStr">
+        <is>
+          <t>Ancien seuil étude (+1.5 m) — référence</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="n">
+      <c r="A17" s="31" t="n">
         <v>37.4</v>
       </c>
       <c r="B17" s="10" t="n">
-        <v>1516</v>
-      </c>
-      <c r="C17" s="28">
+        <v>2320</v>
+      </c>
+      <c r="C17" s="31">
         <f>A17-A16</f>
         <v/>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="32">
         <f>0.5*(B16+B17)*C17</f>
         <v/>
       </c>
-      <c r="E17" s="24">
+      <c r="E17" s="32">
         <f>E16+D17</f>
         <v/>
       </c>
-      <c r="F17" s="26" t="inlineStr">
-        <is>
-          <t>Placeholder — remplacer</t>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>LIMITE VILLE (WSE max + freeboard 0.6 m)</t>
         </is>
       </c>
     </row>
@@ -5152,7 +5183,7 @@
         <v>40</v>
       </c>
       <c r="B18" s="10" t="n">
-        <v>3746</v>
+        <v>3732</v>
       </c>
       <c r="C18" s="28">
         <f>A18-A17</f>
@@ -5168,7 +5199,7 @@
       </c>
       <c r="F18" s="26" t="inlineStr">
         <is>
-          <t>Placeholder haut — remplacer</t>
+          <t>Sommet table</t>
         </is>
       </c>
     </row>
@@ -5205,12 +5236,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>V @ 37.28 m</t>
+          <t>V @ 37.28 m (ancien seuil)</t>
         </is>
       </c>
       <c r="B23" s="34">
         <f>E16</f>
         <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>V @ 37.40 m (limite ville)</t>
+        </is>
+      </c>
+      <c r="B24" s="23">
+        <f>E17</f>
+        <v/>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Comparer a Vmax Methode C</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -5234,14 +5281,14 @@
     <row r="1">
       <c r="A1" s="16" t="inlineStr">
         <is>
-          <t>Methode C — Q_1200 + Q_overflow; V_pond + V_ditch</t>
+          <t>Methode C — Q_1200 + Q_overflow; V = V_pond (+ V_ditch si B25=1)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Lie a Parametres (crest, b, n, z, S, L). Overflow si WSE &gt;= crest.</t>
+          <t>Lie a Parametres B25–B32. Q_overflow si WSE&gt;=crest. B25=0 → V_ditch=0 (leve seul).</t>
         </is>
       </c>
     </row>
@@ -5319,6 +5366,17 @@
       </c>
       <c r="B10" s="27">
         <f>Parametres!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Inclure V_ditch</t>
+        </is>
+      </c>
+      <c r="B11" s="27">
+        <f>Parametres!B25</f>
         <v/>
       </c>
     </row>
@@ -5391,7 +5449,7 @@
         <v/>
       </c>
       <c r="E13" s="18">
-        <f>D13*$B$9</f>
+        <f>IF($B$11=1,D13*$B$9,0)</f>
         <v/>
       </c>
       <c r="F13" s="18">
@@ -5399,7 +5457,7 @@
         <v/>
       </c>
       <c r="G13" s="24">
-        <f>E13+F13</f>
+        <f>F13+E13</f>
         <v/>
       </c>
       <c r="H13" s="19">
@@ -5432,7 +5490,7 @@
         <v/>
       </c>
       <c r="E14" s="18">
-        <f>D14*$B$9</f>
+        <f>IF($B$11=1,D14*$B$9,0)</f>
         <v/>
       </c>
       <c r="F14" s="18">
@@ -5440,7 +5498,7 @@
         <v/>
       </c>
       <c r="G14" s="24">
-        <f>E14+F14</f>
+        <f>F14+E14</f>
         <v/>
       </c>
       <c r="H14" s="19">
@@ -5473,7 +5531,7 @@
         <v/>
       </c>
       <c r="E15" s="18">
-        <f>D15*$B$9</f>
+        <f>IF($B$11=1,D15*$B$9,0)</f>
         <v/>
       </c>
       <c r="F15" s="18">
@@ -5481,7 +5539,7 @@
         <v/>
       </c>
       <c r="G15" s="24">
-        <f>E15+F15</f>
+        <f>F15+E15</f>
         <v/>
       </c>
       <c r="H15" s="19">
@@ -5514,7 +5572,7 @@
         <v/>
       </c>
       <c r="E16" s="18">
-        <f>D16*$B$9</f>
+        <f>IF($B$11=1,D16*$B$9,0)</f>
         <v/>
       </c>
       <c r="F16" s="18">
@@ -5522,7 +5580,7 @@
         <v/>
       </c>
       <c r="G16" s="24">
-        <f>E16+F16</f>
+        <f>F16+E16</f>
         <v/>
       </c>
       <c r="H16" s="19">
@@ -5555,7 +5613,7 @@
         <v/>
       </c>
       <c r="E17" s="18">
-        <f>D17*$B$9</f>
+        <f>IF($B$11=1,D17*$B$9,0)</f>
         <v/>
       </c>
       <c r="F17" s="18">
@@ -5563,7 +5621,7 @@
         <v/>
       </c>
       <c r="G17" s="24">
-        <f>E17+F17</f>
+        <f>F17+E17</f>
         <v/>
       </c>
       <c r="H17" s="19">
@@ -5596,7 +5654,7 @@
         <v/>
       </c>
       <c r="E18" s="18">
-        <f>D18*$B$9</f>
+        <f>IF($B$11=1,D18*$B$9,0)</f>
         <v/>
       </c>
       <c r="F18" s="18">
@@ -5604,7 +5662,7 @@
         <v/>
       </c>
       <c r="G18" s="24">
-        <f>E18+F18</f>
+        <f>F18+E18</f>
         <v/>
       </c>
       <c r="H18" s="19">
@@ -5637,7 +5695,7 @@
         <v/>
       </c>
       <c r="E19" s="18">
-        <f>D19*$B$9</f>
+        <f>IF($B$11=1,D19*$B$9,0)</f>
         <v/>
       </c>
       <c r="F19" s="18">
@@ -5645,7 +5703,7 @@
         <v/>
       </c>
       <c r="G19" s="24">
-        <f>E19+F19</f>
+        <f>F19+E19</f>
         <v/>
       </c>
       <c r="H19" s="19">
@@ -5678,7 +5736,7 @@
         <v/>
       </c>
       <c r="E20" s="18">
-        <f>D20*$B$9</f>
+        <f>IF($B$11=1,D20*$B$9,0)</f>
         <v/>
       </c>
       <c r="F20" s="18">
@@ -5686,7 +5744,7 @@
         <v/>
       </c>
       <c r="G20" s="24">
-        <f>E20+F20</f>
+        <f>F20+E20</f>
         <v/>
       </c>
       <c r="H20" s="19">
@@ -5719,7 +5777,7 @@
         <v/>
       </c>
       <c r="E21" s="18">
-        <f>D21*$B$9</f>
+        <f>IF($B$11=1,D21*$B$9,0)</f>
         <v/>
       </c>
       <c r="F21" s="18">
@@ -5727,7 +5785,7 @@
         <v/>
       </c>
       <c r="G21" s="24">
-        <f>E21+F21</f>
+        <f>F21+E21</f>
         <v/>
       </c>
       <c r="H21" s="19">
@@ -5760,7 +5818,7 @@
         <v/>
       </c>
       <c r="E22" s="18">
-        <f>D22*$B$9</f>
+        <f>IF($B$11=1,D22*$B$9,0)</f>
         <v/>
       </c>
       <c r="F22" s="18">
@@ -5768,7 +5826,7 @@
         <v/>
       </c>
       <c r="G22" s="24">
-        <f>E22+F22</f>
+        <f>F22+E22</f>
         <v/>
       </c>
       <c r="H22" s="19">
@@ -5801,7 +5859,7 @@
         <v/>
       </c>
       <c r="E23" s="18">
-        <f>D23*$B$9</f>
+        <f>IF($B$11=1,D23*$B$9,0)</f>
         <v/>
       </c>
       <c r="F23" s="18">
@@ -5809,7 +5867,7 @@
         <v/>
       </c>
       <c r="G23" s="24">
-        <f>E23+F23</f>
+        <f>F23+E23</f>
         <v/>
       </c>
       <c r="H23" s="19">
@@ -5842,7 +5900,7 @@
         <v/>
       </c>
       <c r="E24" s="18">
-        <f>D24*$B$9</f>
+        <f>IF($B$11=1,D24*$B$9,0)</f>
         <v/>
       </c>
       <c r="F24" s="18">
@@ -5850,7 +5908,7 @@
         <v/>
       </c>
       <c r="G24" s="24">
-        <f>E24+F24</f>
+        <f>F24+E24</f>
         <v/>
       </c>
       <c r="H24" s="19">
@@ -5883,7 +5941,7 @@
         <v/>
       </c>
       <c r="E25" s="18">
-        <f>D25*$B$9</f>
+        <f>IF($B$11=1,D25*$B$9,0)</f>
         <v/>
       </c>
       <c r="F25" s="18">
@@ -5891,7 +5949,7 @@
         <v/>
       </c>
       <c r="G25" s="24">
-        <f>E25+F25</f>
+        <f>F25+E25</f>
         <v/>
       </c>
       <c r="H25" s="19">
@@ -5924,7 +5982,7 @@
         <v/>
       </c>
       <c r="E26" s="18">
-        <f>D26*$B$9</f>
+        <f>IF($B$11=1,D26*$B$9,0)</f>
         <v/>
       </c>
       <c r="F26" s="18">
@@ -5932,7 +5990,7 @@
         <v/>
       </c>
       <c r="G26" s="24">
-        <f>E26+F26</f>
+        <f>F26+E26</f>
         <v/>
       </c>
       <c r="H26" s="19">
@@ -5965,7 +6023,7 @@
         <v/>
       </c>
       <c r="E27" s="18">
-        <f>D27*$B$9</f>
+        <f>IF($B$11=1,D27*$B$9,0)</f>
         <v/>
       </c>
       <c r="F27" s="18">
@@ -5973,7 +6031,7 @@
         <v/>
       </c>
       <c r="G27" s="24">
-        <f>E27+F27</f>
+        <f>F27+E27</f>
         <v/>
       </c>
       <c r="H27" s="19">
@@ -6006,7 +6064,7 @@
         <v/>
       </c>
       <c r="E28" s="18">
-        <f>D28*$B$9</f>
+        <f>IF($B$11=1,D28*$B$9,0)</f>
         <v/>
       </c>
       <c r="F28" s="18">
@@ -6014,7 +6072,7 @@
         <v/>
       </c>
       <c r="G28" s="24">
-        <f>E28+F28</f>
+        <f>F28+E28</f>
         <v/>
       </c>
       <c r="H28" s="19">
@@ -6047,7 +6105,7 @@
         <v/>
       </c>
       <c r="E29" s="18">
-        <f>D29*$B$9</f>
+        <f>IF($B$11=1,D29*$B$9,0)</f>
         <v/>
       </c>
       <c r="F29" s="18">
@@ -6055,7 +6113,7 @@
         <v/>
       </c>
       <c r="G29" s="24">
-        <f>E29+F29</f>
+        <f>F29+E29</f>
         <v/>
       </c>
       <c r="H29" s="19">
@@ -6088,7 +6146,7 @@
         <v/>
       </c>
       <c r="E30" s="18">
-        <f>D30*$B$9</f>
+        <f>IF($B$11=1,D30*$B$9,0)</f>
         <v/>
       </c>
       <c r="F30" s="18">
@@ -6096,7 +6154,7 @@
         <v/>
       </c>
       <c r="G30" s="24">
-        <f>E30+F30</f>
+        <f>F30+E30</f>
         <v/>
       </c>
       <c r="H30" s="19">
@@ -6129,7 +6187,7 @@
         <v/>
       </c>
       <c r="E31" s="18">
-        <f>D31*$B$9</f>
+        <f>IF($B$11=1,D31*$B$9,0)</f>
         <v/>
       </c>
       <c r="F31" s="18">
@@ -6137,7 +6195,7 @@
         <v/>
       </c>
       <c r="G31" s="24">
-        <f>E31+F31</f>
+        <f>F31+E31</f>
         <v/>
       </c>
       <c r="H31" s="19">
@@ -6170,7 +6228,7 @@
         <v/>
       </c>
       <c r="E32" s="18">
-        <f>D32*$B$9</f>
+        <f>IF($B$11=1,D32*$B$9,0)</f>
         <v/>
       </c>
       <c r="F32" s="18">
@@ -6178,7 +6236,7 @@
         <v/>
       </c>
       <c r="G32" s="24">
-        <f>E32+F32</f>
+        <f>F32+E32</f>
         <v/>
       </c>
       <c r="H32" s="19">
@@ -6211,7 +6269,7 @@
         <v/>
       </c>
       <c r="E33" s="18">
-        <f>D33*$B$9</f>
+        <f>IF($B$11=1,D33*$B$9,0)</f>
         <v/>
       </c>
       <c r="F33" s="18">
@@ -6219,7 +6277,7 @@
         <v/>
       </c>
       <c r="G33" s="24">
-        <f>E33+F33</f>
+        <f>F33+E33</f>
         <v/>
       </c>
       <c r="H33" s="19">
@@ -6252,7 +6310,7 @@
         <v/>
       </c>
       <c r="E34" s="18">
-        <f>D34*$B$9</f>
+        <f>IF($B$11=1,D34*$B$9,0)</f>
         <v/>
       </c>
       <c r="F34" s="18">
@@ -6260,7 +6318,7 @@
         <v/>
       </c>
       <c r="G34" s="24">
-        <f>E34+F34</f>
+        <f>F34+E34</f>
         <v/>
       </c>
       <c r="H34" s="19">
@@ -6293,7 +6351,7 @@
         <v/>
       </c>
       <c r="E35" s="18">
-        <f>D35*$B$9</f>
+        <f>IF($B$11=1,D35*$B$9,0)</f>
         <v/>
       </c>
       <c r="F35" s="18">
@@ -6301,7 +6359,7 @@
         <v/>
       </c>
       <c r="G35" s="24">
-        <f>E35+F35</f>
+        <f>F35+E35</f>
         <v/>
       </c>
       <c r="H35" s="19">
@@ -6334,7 +6392,7 @@
         <v/>
       </c>
       <c r="E36" s="18">
-        <f>D36*$B$9</f>
+        <f>IF($B$11=1,D36*$B$9,0)</f>
         <v/>
       </c>
       <c r="F36" s="18">
@@ -6342,7 +6400,7 @@
         <v/>
       </c>
       <c r="G36" s="24">
-        <f>E36+F36</f>
+        <f>F36+E36</f>
         <v/>
       </c>
       <c r="H36" s="19">
@@ -6375,7 +6433,7 @@
         <v/>
       </c>
       <c r="E37" s="18">
-        <f>D37*$B$9</f>
+        <f>IF($B$11=1,D37*$B$9,0)</f>
         <v/>
       </c>
       <c r="F37" s="18">
@@ -6383,7 +6441,7 @@
         <v/>
       </c>
       <c r="G37" s="24">
-        <f>E37+F37</f>
+        <f>F37+E37</f>
         <v/>
       </c>
       <c r="H37" s="19">
@@ -6416,7 +6474,7 @@
         <v/>
       </c>
       <c r="E38" s="18">
-        <f>D38*$B$9</f>
+        <f>IF($B$11=1,D38*$B$9,0)</f>
         <v/>
       </c>
       <c r="F38" s="18">
@@ -6424,7 +6482,7 @@
         <v/>
       </c>
       <c r="G38" s="24">
-        <f>E38+F38</f>
+        <f>F38+E38</f>
         <v/>
       </c>
       <c r="H38" s="19">
@@ -6457,7 +6515,7 @@
         <v/>
       </c>
       <c r="E39" s="18">
-        <f>D39*$B$9</f>
+        <f>IF($B$11=1,D39*$B$9,0)</f>
         <v/>
       </c>
       <c r="F39" s="18">
@@ -6465,7 +6523,7 @@
         <v/>
       </c>
       <c r="G39" s="24">
-        <f>E39+F39</f>
+        <f>F39+E39</f>
         <v/>
       </c>
       <c r="H39" s="19">
@@ -6498,7 +6556,7 @@
         <v/>
       </c>
       <c r="E40" s="18">
-        <f>D40*$B$9</f>
+        <f>IF($B$11=1,D40*$B$9,0)</f>
         <v/>
       </c>
       <c r="F40" s="18">
@@ -6506,7 +6564,7 @@
         <v/>
       </c>
       <c r="G40" s="24">
-        <f>E40+F40</f>
+        <f>F40+E40</f>
         <v/>
       </c>
       <c r="H40" s="19">
@@ -6539,7 +6597,7 @@
         <v/>
       </c>
       <c r="E41" s="18">
-        <f>D41*$B$9</f>
+        <f>IF($B$11=1,D41*$B$9,0)</f>
         <v/>
       </c>
       <c r="F41" s="18">
@@ -6547,7 +6605,7 @@
         <v/>
       </c>
       <c r="G41" s="24">
-        <f>E41+F41</f>
+        <f>F41+E41</f>
         <v/>
       </c>
       <c r="H41" s="19">
@@ -6580,7 +6638,7 @@
         <v/>
       </c>
       <c r="E42" s="18">
-        <f>D42*$B$9</f>
+        <f>IF($B$11=1,D42*$B$9,0)</f>
         <v/>
       </c>
       <c r="F42" s="18">
@@ -6588,7 +6646,7 @@
         <v/>
       </c>
       <c r="G42" s="24">
-        <f>E42+F42</f>
+        <f>F42+E42</f>
         <v/>
       </c>
       <c r="H42" s="19">
@@ -6621,7 +6679,7 @@
         <v/>
       </c>
       <c r="E43" s="18">
-        <f>D43*$B$9</f>
+        <f>IF($B$11=1,D43*$B$9,0)</f>
         <v/>
       </c>
       <c r="F43" s="18">
@@ -6629,7 +6687,7 @@
         <v/>
       </c>
       <c r="G43" s="24">
-        <f>E43+F43</f>
+        <f>F43+E43</f>
         <v/>
       </c>
       <c r="H43" s="19">
@@ -6662,7 +6720,7 @@
         <v/>
       </c>
       <c r="E44" s="18">
-        <f>D44*$B$9</f>
+        <f>IF($B$11=1,D44*$B$9,0)</f>
         <v/>
       </c>
       <c r="F44" s="18">
@@ -6670,7 +6728,7 @@
         <v/>
       </c>
       <c r="G44" s="24">
-        <f>E44+F44</f>
+        <f>F44+E44</f>
         <v/>
       </c>
       <c r="H44" s="19">
@@ -6703,7 +6761,7 @@
         <v/>
       </c>
       <c r="E45" s="18">
-        <f>D45*$B$9</f>
+        <f>IF($B$11=1,D45*$B$9,0)</f>
         <v/>
       </c>
       <c r="F45" s="18">
@@ -6711,7 +6769,7 @@
         <v/>
       </c>
       <c r="G45" s="24">
-        <f>E45+F45</f>
+        <f>F45+E45</f>
         <v/>
       </c>
       <c r="H45" s="19">
@@ -6744,7 +6802,7 @@
         <v/>
       </c>
       <c r="E46" s="18">
-        <f>D46*$B$9</f>
+        <f>IF($B$11=1,D46*$B$9,0)</f>
         <v/>
       </c>
       <c r="F46" s="18">
@@ -6752,7 +6810,7 @@
         <v/>
       </c>
       <c r="G46" s="24">
-        <f>E46+F46</f>
+        <f>F46+E46</f>
         <v/>
       </c>
       <c r="H46" s="19">
@@ -6785,7 +6843,7 @@
         <v/>
       </c>
       <c r="E47" s="18">
-        <f>D47*$B$9</f>
+        <f>IF($B$11=1,D47*$B$9,0)</f>
         <v/>
       </c>
       <c r="F47" s="18">
@@ -6793,7 +6851,7 @@
         <v/>
       </c>
       <c r="G47" s="24">
-        <f>E47+F47</f>
+        <f>F47+E47</f>
         <v/>
       </c>
       <c r="H47" s="19">
@@ -6826,7 +6884,7 @@
         <v/>
       </c>
       <c r="E48" s="18">
-        <f>D48*$B$9</f>
+        <f>IF($B$11=1,D48*$B$9,0)</f>
         <v/>
       </c>
       <c r="F48" s="18">
@@ -6834,7 +6892,7 @@
         <v/>
       </c>
       <c r="G48" s="24">
-        <f>E48+F48</f>
+        <f>F48+E48</f>
         <v/>
       </c>
       <c r="H48" s="19">
@@ -6867,7 +6925,7 @@
         <v/>
       </c>
       <c r="E49" s="18">
-        <f>D49*$B$9</f>
+        <f>IF($B$11=1,D49*$B$9,0)</f>
         <v/>
       </c>
       <c r="F49" s="18">
@@ -6875,7 +6933,7 @@
         <v/>
       </c>
       <c r="G49" s="24">
-        <f>E49+F49</f>
+        <f>F49+E49</f>
         <v/>
       </c>
       <c r="H49" s="19">
@@ -6908,7 +6966,7 @@
         <v/>
       </c>
       <c r="E50" s="18">
-        <f>D50*$B$9</f>
+        <f>IF($B$11=1,D50*$B$9,0)</f>
         <v/>
       </c>
       <c r="F50" s="18">
@@ -6916,7 +6974,7 @@
         <v/>
       </c>
       <c r="G50" s="24">
-        <f>E50+F50</f>
+        <f>F50+E50</f>
         <v/>
       </c>
       <c r="H50" s="19">
@@ -6949,7 +7007,7 @@
         <v/>
       </c>
       <c r="E51" s="18">
-        <f>D51*$B$9</f>
+        <f>IF($B$11=1,D51*$B$9,0)</f>
         <v/>
       </c>
       <c r="F51" s="18">
@@ -6957,7 +7015,7 @@
         <v/>
       </c>
       <c r="G51" s="24">
-        <f>E51+F51</f>
+        <f>F51+E51</f>
         <v/>
       </c>
       <c r="H51" s="19">
@@ -6990,7 +7048,7 @@
         <v/>
       </c>
       <c r="E52" s="18">
-        <f>D52*$B$9</f>
+        <f>IF($B$11=1,D52*$B$9,0)</f>
         <v/>
       </c>
       <c r="F52" s="18">
@@ -6998,7 +7056,7 @@
         <v/>
       </c>
       <c r="G52" s="24">
-        <f>E52+F52</f>
+        <f>F52+E52</f>
         <v/>
       </c>
       <c r="H52" s="19">
@@ -7031,7 +7089,7 @@
         <v/>
       </c>
       <c r="E53" s="18">
-        <f>D53*$B$9</f>
+        <f>IF($B$11=1,D53*$B$9,0)</f>
         <v/>
       </c>
       <c r="F53" s="18">
@@ -7039,7 +7097,7 @@
         <v/>
       </c>
       <c r="G53" s="24">
-        <f>E53+F53</f>
+        <f>F53+E53</f>
         <v/>
       </c>
       <c r="H53" s="19">
@@ -7072,7 +7130,7 @@
         <v/>
       </c>
       <c r="E54" s="18">
-        <f>D54*$B$9</f>
+        <f>IF($B$11=1,D54*$B$9,0)</f>
         <v/>
       </c>
       <c r="F54" s="18">
@@ -7080,7 +7138,7 @@
         <v/>
       </c>
       <c r="G54" s="24">
-        <f>E54+F54</f>
+        <f>F54+E54</f>
         <v/>
       </c>
       <c r="H54" s="19">
@@ -7113,7 +7171,7 @@
         <v/>
       </c>
       <c r="E55" s="18">
-        <f>D55*$B$9</f>
+        <f>IF($B$11=1,D55*$B$9,0)</f>
         <v/>
       </c>
       <c r="F55" s="18">
@@ -7121,7 +7179,7 @@
         <v/>
       </c>
       <c r="G55" s="24">
-        <f>E55+F55</f>
+        <f>F55+E55</f>
         <v/>
       </c>
       <c r="H55" s="19">
@@ -7154,7 +7212,7 @@
         <v/>
       </c>
       <c r="E56" s="18">
-        <f>D56*$B$9</f>
+        <f>IF($B$11=1,D56*$B$9,0)</f>
         <v/>
       </c>
       <c r="F56" s="18">
@@ -7162,7 +7220,7 @@
         <v/>
       </c>
       <c r="G56" s="24">
-        <f>E56+F56</f>
+        <f>F56+E56</f>
         <v/>
       </c>
       <c r="H56" s="19">
@@ -7195,7 +7253,7 @@
         <v/>
       </c>
       <c r="E57" s="18">
-        <f>D57*$B$9</f>
+        <f>IF($B$11=1,D57*$B$9,0)</f>
         <v/>
       </c>
       <c r="F57" s="18">
@@ -7203,7 +7261,7 @@
         <v/>
       </c>
       <c r="G57" s="24">
-        <f>E57+F57</f>
+        <f>F57+E57</f>
         <v/>
       </c>
       <c r="H57" s="19">
@@ -7236,7 +7294,7 @@
         <v/>
       </c>
       <c r="E58" s="18">
-        <f>D58*$B$9</f>
+        <f>IF($B$11=1,D58*$B$9,0)</f>
         <v/>
       </c>
       <c r="F58" s="18">
@@ -7244,7 +7302,7 @@
         <v/>
       </c>
       <c r="G58" s="24">
-        <f>E58+F58</f>
+        <f>F58+E58</f>
         <v/>
       </c>
       <c r="H58" s="19">
@@ -7277,7 +7335,7 @@
         <v/>
       </c>
       <c r="E59" s="18">
-        <f>D59*$B$9</f>
+        <f>IF($B$11=1,D59*$B$9,0)</f>
         <v/>
       </c>
       <c r="F59" s="18">
@@ -7285,7 +7343,7 @@
         <v/>
       </c>
       <c r="G59" s="24">
-        <f>E59+F59</f>
+        <f>F59+E59</f>
         <v/>
       </c>
       <c r="H59" s="19">
@@ -7318,7 +7376,7 @@
         <v/>
       </c>
       <c r="E60" s="18">
-        <f>D60*$B$9</f>
+        <f>IF($B$11=1,D60*$B$9,0)</f>
         <v/>
       </c>
       <c r="F60" s="18">
@@ -7326,7 +7384,7 @@
         <v/>
       </c>
       <c r="G60" s="24">
-        <f>E60+F60</f>
+        <f>F60+E60</f>
         <v/>
       </c>
       <c r="H60" s="19">
@@ -7359,7 +7417,7 @@
         <v/>
       </c>
       <c r="E61" s="18">
-        <f>D61*$B$9</f>
+        <f>IF($B$11=1,D61*$B$9,0)</f>
         <v/>
       </c>
       <c r="F61" s="18">
@@ -7367,7 +7425,7 @@
         <v/>
       </c>
       <c r="G61" s="24">
-        <f>E61+F61</f>
+        <f>F61+E61</f>
         <v/>
       </c>
       <c r="H61" s="19">
@@ -7400,7 +7458,7 @@
         <v/>
       </c>
       <c r="E62" s="18">
-        <f>D62*$B$9</f>
+        <f>IF($B$11=1,D62*$B$9,0)</f>
         <v/>
       </c>
       <c r="F62" s="18">
@@ -7408,7 +7466,7 @@
         <v/>
       </c>
       <c r="G62" s="24">
-        <f>E62+F62</f>
+        <f>F62+E62</f>
         <v/>
       </c>
       <c r="H62" s="19">
@@ -7441,7 +7499,7 @@
         <v/>
       </c>
       <c r="E63" s="18">
-        <f>D63*$B$9</f>
+        <f>IF($B$11=1,D63*$B$9,0)</f>
         <v/>
       </c>
       <c r="F63" s="18">
@@ -7449,7 +7507,7 @@
         <v/>
       </c>
       <c r="G63" s="24">
-        <f>E63+F63</f>
+        <f>F63+E63</f>
         <v/>
       </c>
       <c r="H63" s="19">
@@ -7482,7 +7540,7 @@
         <v/>
       </c>
       <c r="E64" s="18">
-        <f>D64*$B$9</f>
+        <f>IF($B$11=1,D64*$B$9,0)</f>
         <v/>
       </c>
       <c r="F64" s="18">
@@ -7490,7 +7548,7 @@
         <v/>
       </c>
       <c r="G64" s="24">
-        <f>E64+F64</f>
+        <f>F64+E64</f>
         <v/>
       </c>
       <c r="H64" s="19">
@@ -7534,7 +7592,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>WSE depuis V_total (Compose_1200); Qout = Q_1200 + Q_overflow.</t>
+          <t>WSE depuis V_total (Compose_1200; B25 pilote V_ditch). Qout = Q_1200 + Q_overflow.</t>
         </is>
       </c>
     </row>
@@ -8042,7 +8100,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>1. Le Ø900 est elimine: plus de controle etroit; le bassin peut etre agrandi (Stage_Storage).</t>
+          <t>1. Le Ø900 est elimine: controle = Ø1200; Stage_Storage = aires Z1+Z2 (leve combine).</t>
         </is>
       </c>
     </row>
@@ -8077,7 +8135,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t xml:space="preserve">   C) Qout = Q_1200 + overflow trapèze au-dessus du crest (berme/fosse).</t>
+          <t xml:space="preserve">   C) Qout = Q_1200 + Q_overflow; V = leve (+ V_ditch si Parametres B25=1).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Sans_900 overflow velocity artifacts
Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
@@ -6213,7 +6213,7 @@
         <v/>
       </c>
       <c r="L13" s="20">
-        <f>IF(D13&lt;=0,0,I13/D13)</f>
+        <f>IF(OR(C13&lt;0.05,D13&lt;0.05),"",I13/D13)</f>
         <v/>
       </c>
     </row>
@@ -6262,7 +6262,7 @@
         <v/>
       </c>
       <c r="L14" s="20">
-        <f>IF(D14&lt;=0,0,I14/D14)</f>
+        <f>IF(OR(C14&lt;0.05,D14&lt;0.05),"",I14/D14)</f>
         <v/>
       </c>
     </row>
@@ -6311,7 +6311,7 @@
         <v/>
       </c>
       <c r="L15" s="20">
-        <f>IF(D15&lt;=0,0,I15/D15)</f>
+        <f>IF(OR(C15&lt;0.05,D15&lt;0.05),"",I15/D15)</f>
         <v/>
       </c>
     </row>
@@ -6360,7 +6360,7 @@
         <v/>
       </c>
       <c r="L16" s="20">
-        <f>IF(D16&lt;=0,0,I16/D16)</f>
+        <f>IF(OR(C16&lt;0.05,D16&lt;0.05),"",I16/D16)</f>
         <v/>
       </c>
     </row>
@@ -6409,7 +6409,7 @@
         <v/>
       </c>
       <c r="L17" s="20">
-        <f>IF(D17&lt;=0,0,I17/D17)</f>
+        <f>IF(OR(C17&lt;0.05,D17&lt;0.05),"",I17/D17)</f>
         <v/>
       </c>
     </row>
@@ -6458,7 +6458,7 @@
         <v/>
       </c>
       <c r="L18" s="20">
-        <f>IF(D18&lt;=0,0,I18/D18)</f>
+        <f>IF(OR(C18&lt;0.05,D18&lt;0.05),"",I18/D18)</f>
         <v/>
       </c>
     </row>
@@ -6507,7 +6507,7 @@
         <v/>
       </c>
       <c r="L19" s="20">
-        <f>IF(D19&lt;=0,0,I19/D19)</f>
+        <f>IF(OR(C19&lt;0.05,D19&lt;0.05),"",I19/D19)</f>
         <v/>
       </c>
     </row>
@@ -6556,7 +6556,7 @@
         <v/>
       </c>
       <c r="L20" s="20">
-        <f>IF(D20&lt;=0,0,I20/D20)</f>
+        <f>IF(OR(C20&lt;0.05,D20&lt;0.05),"",I20/D20)</f>
         <v/>
       </c>
     </row>
@@ -6605,7 +6605,7 @@
         <v/>
       </c>
       <c r="L21" s="20">
-        <f>IF(D21&lt;=0,0,I21/D21)</f>
+        <f>IF(OR(C21&lt;0.05,D21&lt;0.05),"",I21/D21)</f>
         <v/>
       </c>
     </row>
@@ -6654,7 +6654,7 @@
         <v/>
       </c>
       <c r="L22" s="20">
-        <f>IF(D22&lt;=0,0,I22/D22)</f>
+        <f>IF(OR(C22&lt;0.05,D22&lt;0.05),"",I22/D22)</f>
         <v/>
       </c>
     </row>
@@ -6703,7 +6703,7 @@
         <v/>
       </c>
       <c r="L23" s="20">
-        <f>IF(D23&lt;=0,0,I23/D23)</f>
+        <f>IF(OR(C23&lt;0.05,D23&lt;0.05),"",I23/D23)</f>
         <v/>
       </c>
     </row>
@@ -6752,7 +6752,7 @@
         <v/>
       </c>
       <c r="L24" s="20">
-        <f>IF(D24&lt;=0,0,I24/D24)</f>
+        <f>IF(OR(C24&lt;0.05,D24&lt;0.05),"",I24/D24)</f>
         <v/>
       </c>
     </row>
@@ -6801,7 +6801,7 @@
         <v/>
       </c>
       <c r="L25" s="20">
-        <f>IF(D25&lt;=0,0,I25/D25)</f>
+        <f>IF(OR(C25&lt;0.05,D25&lt;0.05),"",I25/D25)</f>
         <v/>
       </c>
     </row>
@@ -6850,7 +6850,7 @@
         <v/>
       </c>
       <c r="L26" s="20">
-        <f>IF(D26&lt;=0,0,I26/D26)</f>
+        <f>IF(OR(C26&lt;0.05,D26&lt;0.05),"",I26/D26)</f>
         <v/>
       </c>
     </row>
@@ -6899,7 +6899,7 @@
         <v/>
       </c>
       <c r="L27" s="20">
-        <f>IF(D27&lt;=0,0,I27/D27)</f>
+        <f>IF(OR(C27&lt;0.05,D27&lt;0.05),"",I27/D27)</f>
         <v/>
       </c>
     </row>
@@ -6948,7 +6948,7 @@
         <v/>
       </c>
       <c r="L28" s="20">
-        <f>IF(D28&lt;=0,0,I28/D28)</f>
+        <f>IF(OR(C28&lt;0.05,D28&lt;0.05),"",I28/D28)</f>
         <v/>
       </c>
     </row>
@@ -6997,7 +6997,7 @@
         <v/>
       </c>
       <c r="L29" s="20">
-        <f>IF(D29&lt;=0,0,I29/D29)</f>
+        <f>IF(OR(C29&lt;0.05,D29&lt;0.05),"",I29/D29)</f>
         <v/>
       </c>
     </row>
@@ -7046,7 +7046,7 @@
         <v/>
       </c>
       <c r="L30" s="20">
-        <f>IF(D30&lt;=0,0,I30/D30)</f>
+        <f>IF(OR(C30&lt;0.05,D30&lt;0.05),"",I30/D30)</f>
         <v/>
       </c>
     </row>
@@ -7095,7 +7095,7 @@
         <v/>
       </c>
       <c r="L31" s="20">
-        <f>IF(D31&lt;=0,0,I31/D31)</f>
+        <f>IF(OR(C31&lt;0.05,D31&lt;0.05),"",I31/D31)</f>
         <v/>
       </c>
     </row>
@@ -7144,7 +7144,7 @@
         <v/>
       </c>
       <c r="L32" s="20">
-        <f>IF(D32&lt;=0,0,I32/D32)</f>
+        <f>IF(OR(C32&lt;0.05,D32&lt;0.05),"",I32/D32)</f>
         <v/>
       </c>
     </row>
@@ -7193,7 +7193,7 @@
         <v/>
       </c>
       <c r="L33" s="20">
-        <f>IF(D33&lt;=0,0,I33/D33)</f>
+        <f>IF(OR(C33&lt;0.05,D33&lt;0.05),"",I33/D33)</f>
         <v/>
       </c>
     </row>
@@ -7242,7 +7242,7 @@
         <v/>
       </c>
       <c r="L34" s="20">
-        <f>IF(D34&lt;=0,0,I34/D34)</f>
+        <f>IF(OR(C34&lt;0.05,D34&lt;0.05),"",I34/D34)</f>
         <v/>
       </c>
     </row>
@@ -7291,7 +7291,7 @@
         <v/>
       </c>
       <c r="L35" s="20">
-        <f>IF(D35&lt;=0,0,I35/D35)</f>
+        <f>IF(OR(C35&lt;0.05,D35&lt;0.05),"",I35/D35)</f>
         <v/>
       </c>
     </row>
@@ -7340,7 +7340,7 @@
         <v/>
       </c>
       <c r="L36" s="20">
-        <f>IF(D36&lt;=0,0,I36/D36)</f>
+        <f>IF(OR(C36&lt;0.05,D36&lt;0.05),"",I36/D36)</f>
         <v/>
       </c>
     </row>
@@ -7389,7 +7389,7 @@
         <v/>
       </c>
       <c r="L37" s="20">
-        <f>IF(D37&lt;=0,0,I37/D37)</f>
+        <f>IF(OR(C37&lt;0.05,D37&lt;0.05),"",I37/D37)</f>
         <v/>
       </c>
     </row>
@@ -7438,7 +7438,7 @@
         <v/>
       </c>
       <c r="L38" s="20">
-        <f>IF(D38&lt;=0,0,I38/D38)</f>
+        <f>IF(OR(C38&lt;0.05,D38&lt;0.05),"",I38/D38)</f>
         <v/>
       </c>
     </row>
@@ -7487,7 +7487,7 @@
         <v/>
       </c>
       <c r="L39" s="20">
-        <f>IF(D39&lt;=0,0,I39/D39)</f>
+        <f>IF(OR(C39&lt;0.05,D39&lt;0.05),"",I39/D39)</f>
         <v/>
       </c>
     </row>
@@ -7536,7 +7536,7 @@
         <v/>
       </c>
       <c r="L40" s="20">
-        <f>IF(D40&lt;=0,0,I40/D40)</f>
+        <f>IF(OR(C40&lt;0.05,D40&lt;0.05),"",I40/D40)</f>
         <v/>
       </c>
     </row>
@@ -7585,7 +7585,7 @@
         <v/>
       </c>
       <c r="L41" s="20">
-        <f>IF(D41&lt;=0,0,I41/D41)</f>
+        <f>IF(OR(C41&lt;0.05,D41&lt;0.05),"",I41/D41)</f>
         <v/>
       </c>
     </row>
@@ -7634,7 +7634,7 @@
         <v/>
       </c>
       <c r="L42" s="20">
-        <f>IF(D42&lt;=0,0,I42/D42)</f>
+        <f>IF(OR(C42&lt;0.05,D42&lt;0.05),"",I42/D42)</f>
         <v/>
       </c>
     </row>
@@ -7683,7 +7683,7 @@
         <v/>
       </c>
       <c r="L43" s="20">
-        <f>IF(D43&lt;=0,0,I43/D43)</f>
+        <f>IF(OR(C43&lt;0.05,D43&lt;0.05),"",I43/D43)</f>
         <v/>
       </c>
     </row>
@@ -7732,7 +7732,7 @@
         <v/>
       </c>
       <c r="L44" s="20">
-        <f>IF(D44&lt;=0,0,I44/D44)</f>
+        <f>IF(OR(C44&lt;0.05,D44&lt;0.05),"",I44/D44)</f>
         <v/>
       </c>
     </row>
@@ -7781,7 +7781,7 @@
         <v/>
       </c>
       <c r="L45" s="20">
-        <f>IF(D45&lt;=0,0,I45/D45)</f>
+        <f>IF(OR(C45&lt;0.05,D45&lt;0.05),"",I45/D45)</f>
         <v/>
       </c>
     </row>
@@ -7830,7 +7830,7 @@
         <v/>
       </c>
       <c r="L46" s="20">
-        <f>IF(D46&lt;=0,0,I46/D46)</f>
+        <f>IF(OR(C46&lt;0.05,D46&lt;0.05),"",I46/D46)</f>
         <v/>
       </c>
     </row>
@@ -7879,7 +7879,7 @@
         <v/>
       </c>
       <c r="L47" s="20">
-        <f>IF(D47&lt;=0,0,I47/D47)</f>
+        <f>IF(OR(C47&lt;0.05,D47&lt;0.05),"",I47/D47)</f>
         <v/>
       </c>
     </row>
@@ -7928,7 +7928,7 @@
         <v/>
       </c>
       <c r="L48" s="20">
-        <f>IF(D48&lt;=0,0,I48/D48)</f>
+        <f>IF(OR(C48&lt;0.05,D48&lt;0.05),"",I48/D48)</f>
         <v/>
       </c>
     </row>
@@ -7977,7 +7977,7 @@
         <v/>
       </c>
       <c r="L49" s="20">
-        <f>IF(D49&lt;=0,0,I49/D49)</f>
+        <f>IF(OR(C49&lt;0.05,D49&lt;0.05),"",I49/D49)</f>
         <v/>
       </c>
     </row>
@@ -8026,7 +8026,7 @@
         <v/>
       </c>
       <c r="L50" s="20">
-        <f>IF(D50&lt;=0,0,I50/D50)</f>
+        <f>IF(OR(C50&lt;0.05,D50&lt;0.05),"",I50/D50)</f>
         <v/>
       </c>
     </row>
@@ -8075,7 +8075,7 @@
         <v/>
       </c>
       <c r="L51" s="20">
-        <f>IF(D51&lt;=0,0,I51/D51)</f>
+        <f>IF(OR(C51&lt;0.05,D51&lt;0.05),"",I51/D51)</f>
         <v/>
       </c>
     </row>
@@ -8124,7 +8124,7 @@
         <v/>
       </c>
       <c r="L52" s="20">
-        <f>IF(D52&lt;=0,0,I52/D52)</f>
+        <f>IF(OR(C52&lt;0.05,D52&lt;0.05),"",I52/D52)</f>
         <v/>
       </c>
     </row>
@@ -8173,7 +8173,7 @@
         <v/>
       </c>
       <c r="L53" s="20">
-        <f>IF(D53&lt;=0,0,I53/D53)</f>
+        <f>IF(OR(C53&lt;0.05,D53&lt;0.05),"",I53/D53)</f>
         <v/>
       </c>
     </row>
@@ -8222,7 +8222,7 @@
         <v/>
       </c>
       <c r="L54" s="20">
-        <f>IF(D54&lt;=0,0,I54/D54)</f>
+        <f>IF(OR(C54&lt;0.05,D54&lt;0.05),"",I54/D54)</f>
         <v/>
       </c>
     </row>
@@ -8271,7 +8271,7 @@
         <v/>
       </c>
       <c r="L55" s="20">
-        <f>IF(D55&lt;=0,0,I55/D55)</f>
+        <f>IF(OR(C55&lt;0.05,D55&lt;0.05),"",I55/D55)</f>
         <v/>
       </c>
     </row>
@@ -8320,7 +8320,7 @@
         <v/>
       </c>
       <c r="L56" s="20">
-        <f>IF(D56&lt;=0,0,I56/D56)</f>
+        <f>IF(OR(C56&lt;0.05,D56&lt;0.05),"",I56/D56)</f>
         <v/>
       </c>
     </row>
@@ -8369,7 +8369,7 @@
         <v/>
       </c>
       <c r="L57" s="20">
-        <f>IF(D57&lt;=0,0,I57/D57)</f>
+        <f>IF(OR(C57&lt;0.05,D57&lt;0.05),"",I57/D57)</f>
         <v/>
       </c>
     </row>
@@ -8418,7 +8418,7 @@
         <v/>
       </c>
       <c r="L58" s="20">
-        <f>IF(D58&lt;=0,0,I58/D58)</f>
+        <f>IF(OR(C58&lt;0.05,D58&lt;0.05),"",I58/D58)</f>
         <v/>
       </c>
     </row>
@@ -8467,7 +8467,7 @@
         <v/>
       </c>
       <c r="L59" s="20">
-        <f>IF(D59&lt;=0,0,I59/D59)</f>
+        <f>IF(OR(C59&lt;0.05,D59&lt;0.05),"",I59/D59)</f>
         <v/>
       </c>
     </row>
@@ -8516,7 +8516,7 @@
         <v/>
       </c>
       <c r="L60" s="20">
-        <f>IF(D60&lt;=0,0,I60/D60)</f>
+        <f>IF(OR(C60&lt;0.05,D60&lt;0.05),"",I60/D60)</f>
         <v/>
       </c>
     </row>
@@ -8565,7 +8565,7 @@
         <v/>
       </c>
       <c r="L61" s="20">
-        <f>IF(D61&lt;=0,0,I61/D61)</f>
+        <f>IF(OR(C61&lt;0.05,D61&lt;0.05),"",I61/D61)</f>
         <v/>
       </c>
     </row>
@@ -8614,7 +8614,7 @@
         <v/>
       </c>
       <c r="L62" s="20">
-        <f>IF(D62&lt;=0,0,I62/D62)</f>
+        <f>IF(OR(C62&lt;0.05,D62&lt;0.05),"",I62/D62)</f>
         <v/>
       </c>
     </row>
@@ -8663,7 +8663,7 @@
         <v/>
       </c>
       <c r="L63" s="20">
-        <f>IF(D63&lt;=0,0,I63/D63)</f>
+        <f>IF(OR(C63&lt;0.05,D63&lt;0.05),"",I63/D63)</f>
         <v/>
       </c>
     </row>
@@ -8712,7 +8712,7 @@
         <v/>
       </c>
       <c r="L64" s="20">
-        <f>IF(D64&lt;=0,0,I64/D64)</f>
+        <f>IF(OR(C64&lt;0.05,D64&lt;0.05),"",I64/D64)</f>
         <v/>
       </c>
     </row>
@@ -8830,7 +8830,7 @@
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>V_eq_Ø1200 (m/s)</t>
+          <t>V_pipe_seul (m/s)</t>
         </is>
       </c>
     </row>
@@ -8863,7 +8863,7 @@
         </is>
       </c>
       <c r="H10" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D10/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C10&gt;$B$5),"",D10/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
         <v/>
       </c>
       <c r="H11" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D11/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C11&gt;$B$5),"",D11/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -8931,7 +8931,7 @@
         <v/>
       </c>
       <c r="H12" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D12/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C12&gt;$B$5),"",D12/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -8965,7 +8965,7 @@
         <v/>
       </c>
       <c r="H13" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D13/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C13&gt;$B$5),"",D13/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -8999,7 +8999,7 @@
         <v/>
       </c>
       <c r="H14" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D14/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C14&gt;$B$5),"",D14/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9033,7 +9033,7 @@
         <v/>
       </c>
       <c r="H15" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D15/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C15&gt;$B$5),"",D15/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9067,7 +9067,7 @@
         <v/>
       </c>
       <c r="H16" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D16/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C16&gt;$B$5),"",D16/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9101,7 +9101,7 @@
         <v/>
       </c>
       <c r="H17" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D17/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C17&gt;$B$5),"",D17/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9135,7 +9135,7 @@
         <v/>
       </c>
       <c r="H18" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D18/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C18&gt;$B$5),"",D18/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9169,7 +9169,7 @@
         <v/>
       </c>
       <c r="H19" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D19/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C19&gt;$B$5),"",D19/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9203,7 +9203,7 @@
         <v/>
       </c>
       <c r="H20" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D20/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C20&gt;$B$5),"",D20/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9237,7 +9237,7 @@
         <v/>
       </c>
       <c r="H21" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D21/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C21&gt;$B$5),"",D21/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>
@@ -9271,7 +9271,7 @@
         <v/>
       </c>
       <c r="H22" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,D22/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$96&lt;=0,C22&gt;$B$5),"",D22/Parametres!$C$96)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Move Sans_900 velocity table up under Parametres notes
Hard-coding at row 92 left a large empty gap after Notes dynamiques;
table now starts at row 60 and A_plein refs use C64.

Co-authored-by: acon560-prog <acon560-prog@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
+++ b/engineering/drainage-design/retention_volume/Volume_Retention_Sans_900.xlsx
@@ -1683,7 +1683,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F97"/>
+  <dimension ref="A1:F65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -2212,115 +2212,115 @@
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" s="16" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="16" t="inlineStr">
         <is>
           <t>Vitesses de reference — V = Q / A_plein</t>
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
+    <row r="61">
+      <c r="A61" t="inlineStr">
         <is>
           <t>Sans Ø900: control = Ø1200. V_eq = Q/A_plein. Partiellement rempli: V reelle = Q/A(h) plus elevee — voir Courbe_QH_1200.</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="17" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="17" t="inlineStr">
         <is>
           <t>Ouvrage</t>
         </is>
       </c>
-      <c r="B94" s="17" t="inlineStr">
+      <c r="B62" s="17" t="inlineStr">
         <is>
           <t>D (m)</t>
         </is>
       </c>
-      <c r="C94" s="17" t="inlineStr">
+      <c r="C62" s="17" t="inlineStr">
         <is>
           <t>A_plein (m2)</t>
         </is>
       </c>
-      <c r="D94" s="17" t="inlineStr">
+      <c r="D62" s="17" t="inlineStr">
         <is>
           <t>Q ref</t>
         </is>
       </c>
-      <c r="E94" s="17" t="inlineStr">
+      <c r="E62" s="17" t="inlineStr">
         <is>
           <t>V_eq (m/s)</t>
         </is>
       </c>
-      <c r="F94" s="17" t="inlineStr">
+      <c r="F62" s="17" t="inlineStr">
         <is>
           <t>Note</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="18" t="inlineStr">
+    <row r="63">
+      <c r="A63" s="18" t="inlineStr">
         <is>
           <t>Ø1500 (entree)</t>
         </is>
       </c>
-      <c r="B95" s="18" t="n">
+      <c r="B63" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="C95" s="19">
-        <f>PI()*B95^2/4</f>
-        <v/>
-      </c>
-      <c r="D95" s="19">
+      <c r="C63" s="19">
+        <f>PI()*B63^2/4</f>
+        <v/>
+      </c>
+      <c r="D63" s="19">
         <f>Hydrogramme!B4</f>
         <v/>
       </c>
-      <c r="E95" s="20">
-        <f>IF(C95&lt;=0,0,D95/C95)</f>
-        <v/>
-      </c>
-      <c r="F95" s="18" t="inlineStr">
+      <c r="E63" s="20">
+        <f>IF(C63&lt;=0,0,D63/C63)</f>
+        <v/>
+      </c>
+      <c r="F63" s="18" t="inlineStr">
         <is>
           <t>Qpointe</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="18" t="inlineStr">
+    <row r="64">
+      <c r="A64" s="18" t="inlineStr">
         <is>
           <t>Ø1200 (controle)</t>
         </is>
       </c>
-      <c r="B96" s="18">
+      <c r="B64" s="18">
         <f>B11</f>
         <v/>
       </c>
-      <c r="C96" s="19">
+      <c r="C64" s="19">
         <f>B16</f>
         <v/>
       </c>
-      <c r="D96" s="19">
+      <c r="D64" s="19">
         <f>B18</f>
         <v/>
       </c>
-      <c r="E96" s="20">
-        <f>IF(C96&lt;=0,0,D96/C96)</f>
-        <v/>
-      </c>
-      <c r="F96" s="18" t="inlineStr">
+      <c r="E64" s="20">
+        <f>IF(C64&lt;=0,0,D64/C64)</f>
+        <v/>
+      </c>
+      <c r="F64" s="18" t="inlineStr">
         <is>
           <t>Q_plein Manning</t>
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+    <row r="65">
+      <c r="A65" t="inlineStr">
         <is>
           <t>V_Ø1200 @ Qout Calcul_A (m/s)</t>
         </is>
       </c>
-      <c r="B97" s="14">
-        <f>IF(C96&lt;=0,0,Calcul_A!B2/C96)</f>
+      <c r="B65" s="14">
+        <f>IF(C64&lt;=0,0,Calcul_A!B2/C64)</f>
         <v/>
       </c>
     </row>
@@ -2328,8 +2328,8 @@
   <mergeCells count="8">
     <mergeCell ref="A54:F54"/>
     <mergeCell ref="A2:F3"/>
-    <mergeCell ref="A93:F93"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A61:F61"/>
     <mergeCell ref="A58:F58"/>
     <mergeCell ref="A56:F56"/>
     <mergeCell ref="A55:F55"/>
@@ -2712,7 +2712,7 @@
         <v>0</v>
       </c>
       <c r="F8" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C8/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C8/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
         <v/>
       </c>
       <c r="F9" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C9/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C9/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2764,7 +2764,7 @@
         <v/>
       </c>
       <c r="F10" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C10/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C10/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2790,7 +2790,7 @@
         <v/>
       </c>
       <c r="F11" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C11/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C11/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2816,7 +2816,7 @@
         <v/>
       </c>
       <c r="F12" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C12/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C12/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
         <v/>
       </c>
       <c r="F13" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C13/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C13/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
         <v/>
       </c>
       <c r="F14" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C14/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C14/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2894,7 +2894,7 @@
         <v/>
       </c>
       <c r="F15" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C15/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C15/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
         <v/>
       </c>
       <c r="F16" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C16/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C16/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2946,7 +2946,7 @@
         <v/>
       </c>
       <c r="F17" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C17/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C17/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2972,7 +2972,7 @@
         <v/>
       </c>
       <c r="F18" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C18/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C18/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -2998,7 +2998,7 @@
         <v/>
       </c>
       <c r="F19" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C19/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C19/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -3024,7 +3024,7 @@
         <v/>
       </c>
       <c r="F20" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,C20/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,C20/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5247,7 +5247,7 @@
         <v>0</v>
       </c>
       <c r="H10" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E10/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E10/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5281,7 +5281,7 @@
         <v/>
       </c>
       <c r="H11" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E11/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E11/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5315,7 +5315,7 @@
         <v/>
       </c>
       <c r="H12" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E12/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E12/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5349,7 +5349,7 @@
         <v/>
       </c>
       <c r="H13" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E13/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E13/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5383,7 +5383,7 @@
         <v/>
       </c>
       <c r="H14" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E14/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E14/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5417,7 +5417,7 @@
         <v/>
       </c>
       <c r="H15" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E15/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E15/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5451,7 +5451,7 @@
         <v/>
       </c>
       <c r="H16" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E16/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E16/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5485,7 +5485,7 @@
         <v/>
       </c>
       <c r="H17" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E17/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E17/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5519,7 +5519,7 @@
         <v/>
       </c>
       <c r="H18" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E18/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E18/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5553,7 +5553,7 @@
         <v/>
       </c>
       <c r="H19" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E19/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E19/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5587,7 +5587,7 @@
         <v/>
       </c>
       <c r="H20" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E20/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E20/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5621,7 +5621,7 @@
         <v/>
       </c>
       <c r="H21" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E21/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E21/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
         <v/>
       </c>
       <c r="H22" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,E22/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,E22/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="K13" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H13/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H13/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L13" s="20">
@@ -6258,7 +6258,7 @@
         <v/>
       </c>
       <c r="K14" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H14/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H14/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L14" s="20">
@@ -6307,7 +6307,7 @@
         <v/>
       </c>
       <c r="K15" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H15/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H15/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L15" s="20">
@@ -6356,7 +6356,7 @@
         <v/>
       </c>
       <c r="K16" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H16/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H16/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L16" s="20">
@@ -6405,7 +6405,7 @@
         <v/>
       </c>
       <c r="K17" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H17/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H17/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L17" s="20">
@@ -6454,7 +6454,7 @@
         <v/>
       </c>
       <c r="K18" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H18/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H18/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L18" s="20">
@@ -6503,7 +6503,7 @@
         <v/>
       </c>
       <c r="K19" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H19/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H19/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L19" s="20">
@@ -6552,7 +6552,7 @@
         <v/>
       </c>
       <c r="K20" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H20/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H20/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L20" s="20">
@@ -6601,7 +6601,7 @@
         <v/>
       </c>
       <c r="K21" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H21/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H21/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L21" s="20">
@@ -6650,7 +6650,7 @@
         <v/>
       </c>
       <c r="K22" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H22/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H22/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L22" s="20">
@@ -6699,7 +6699,7 @@
         <v/>
       </c>
       <c r="K23" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H23/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H23/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L23" s="20">
@@ -6748,7 +6748,7 @@
         <v/>
       </c>
       <c r="K24" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H24/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H24/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L24" s="20">
@@ -6797,7 +6797,7 @@
         <v/>
       </c>
       <c r="K25" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H25/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H25/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L25" s="20">
@@ -6846,7 +6846,7 @@
         <v/>
       </c>
       <c r="K26" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H26/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H26/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L26" s="20">
@@ -6895,7 +6895,7 @@
         <v/>
       </c>
       <c r="K27" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H27/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H27/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L27" s="20">
@@ -6944,7 +6944,7 @@
         <v/>
       </c>
       <c r="K28" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H28/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H28/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L28" s="20">
@@ -6993,7 +6993,7 @@
         <v/>
       </c>
       <c r="K29" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H29/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H29/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L29" s="20">
@@ -7042,7 +7042,7 @@
         <v/>
       </c>
       <c r="K30" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H30/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H30/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L30" s="20">
@@ -7091,7 +7091,7 @@
         <v/>
       </c>
       <c r="K31" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H31/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H31/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L31" s="20">
@@ -7140,7 +7140,7 @@
         <v/>
       </c>
       <c r="K32" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H32/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H32/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L32" s="20">
@@ -7189,7 +7189,7 @@
         <v/>
       </c>
       <c r="K33" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H33/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H33/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L33" s="20">
@@ -7238,7 +7238,7 @@
         <v/>
       </c>
       <c r="K34" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H34/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H34/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L34" s="20">
@@ -7287,7 +7287,7 @@
         <v/>
       </c>
       <c r="K35" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H35/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H35/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L35" s="20">
@@ -7336,7 +7336,7 @@
         <v/>
       </c>
       <c r="K36" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H36/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H36/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L36" s="20">
@@ -7385,7 +7385,7 @@
         <v/>
       </c>
       <c r="K37" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H37/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H37/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L37" s="20">
@@ -7434,7 +7434,7 @@
         <v/>
       </c>
       <c r="K38" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H38/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H38/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L38" s="20">
@@ -7483,7 +7483,7 @@
         <v/>
       </c>
       <c r="K39" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H39/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H39/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L39" s="20">
@@ -7532,7 +7532,7 @@
         <v/>
       </c>
       <c r="K40" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H40/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H40/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L40" s="20">
@@ -7581,7 +7581,7 @@
         <v/>
       </c>
       <c r="K41" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H41/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H41/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L41" s="20">
@@ -7630,7 +7630,7 @@
         <v/>
       </c>
       <c r="K42" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H42/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H42/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L42" s="20">
@@ -7679,7 +7679,7 @@
         <v/>
       </c>
       <c r="K43" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H43/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H43/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L43" s="20">
@@ -7728,7 +7728,7 @@
         <v/>
       </c>
       <c r="K44" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H44/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H44/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L44" s="20">
@@ -7777,7 +7777,7 @@
         <v/>
       </c>
       <c r="K45" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H45/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H45/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L45" s="20">
@@ -7826,7 +7826,7 @@
         <v/>
       </c>
       <c r="K46" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H46/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H46/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L46" s="20">
@@ -7875,7 +7875,7 @@
         <v/>
       </c>
       <c r="K47" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H47/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H47/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L47" s="20">
@@ -7924,7 +7924,7 @@
         <v/>
       </c>
       <c r="K48" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H48/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H48/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L48" s="20">
@@ -7973,7 +7973,7 @@
         <v/>
       </c>
       <c r="K49" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H49/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H49/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L49" s="20">
@@ -8022,7 +8022,7 @@
         <v/>
       </c>
       <c r="K50" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H50/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H50/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L50" s="20">
@@ -8071,7 +8071,7 @@
         <v/>
       </c>
       <c r="K51" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H51/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H51/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L51" s="20">
@@ -8120,7 +8120,7 @@
         <v/>
       </c>
       <c r="K52" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H52/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H52/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L52" s="20">
@@ -8169,7 +8169,7 @@
         <v/>
       </c>
       <c r="K53" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H53/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H53/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L53" s="20">
@@ -8218,7 +8218,7 @@
         <v/>
       </c>
       <c r="K54" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H54/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H54/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L54" s="20">
@@ -8267,7 +8267,7 @@
         <v/>
       </c>
       <c r="K55" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H55/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H55/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L55" s="20">
@@ -8316,7 +8316,7 @@
         <v/>
       </c>
       <c r="K56" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H56/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H56/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L56" s="20">
@@ -8365,7 +8365,7 @@
         <v/>
       </c>
       <c r="K57" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H57/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H57/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L57" s="20">
@@ -8414,7 +8414,7 @@
         <v/>
       </c>
       <c r="K58" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H58/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H58/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L58" s="20">
@@ -8463,7 +8463,7 @@
         <v/>
       </c>
       <c r="K59" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H59/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H59/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L59" s="20">
@@ -8512,7 +8512,7 @@
         <v/>
       </c>
       <c r="K60" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H60/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H60/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L60" s="20">
@@ -8561,7 +8561,7 @@
         <v/>
       </c>
       <c r="K61" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H61/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H61/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L61" s="20">
@@ -8610,7 +8610,7 @@
         <v/>
       </c>
       <c r="K62" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H62/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H62/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L62" s="20">
@@ -8659,7 +8659,7 @@
         <v/>
       </c>
       <c r="K63" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H63/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H63/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L63" s="20">
@@ -8708,7 +8708,7 @@
         <v/>
       </c>
       <c r="K64" s="20">
-        <f>IF(Parametres!$C$96&lt;=0,0,H64/Parametres!$C$96)</f>
+        <f>IF(Parametres!$C$64&lt;=0,0,H64/Parametres!$C$64)</f>
         <v/>
       </c>
       <c r="L64" s="20">
@@ -8863,7 +8863,7 @@
         </is>
       </c>
       <c r="H10" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C10&gt;$B$5),"",D10/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C10&gt;$B$5),"",D10/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -8897,7 +8897,7 @@
         <v/>
       </c>
       <c r="H11" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C11&gt;$B$5),"",D11/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C11&gt;$B$5),"",D11/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -8931,7 +8931,7 @@
         <v/>
       </c>
       <c r="H12" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C12&gt;$B$5),"",D12/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C12&gt;$B$5),"",D12/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -8965,7 +8965,7 @@
         <v/>
       </c>
       <c r="H13" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C13&gt;$B$5),"",D13/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C13&gt;$B$5),"",D13/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -8999,7 +8999,7 @@
         <v/>
       </c>
       <c r="H14" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C14&gt;$B$5),"",D14/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C14&gt;$B$5),"",D14/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9033,7 +9033,7 @@
         <v/>
       </c>
       <c r="H15" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C15&gt;$B$5),"",D15/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C15&gt;$B$5),"",D15/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9067,7 +9067,7 @@
         <v/>
       </c>
       <c r="H16" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C16&gt;$B$5),"",D16/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C16&gt;$B$5),"",D16/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9101,7 +9101,7 @@
         <v/>
       </c>
       <c r="H17" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C17&gt;$B$5),"",D17/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C17&gt;$B$5),"",D17/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9135,7 +9135,7 @@
         <v/>
       </c>
       <c r="H18" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C18&gt;$B$5),"",D18/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C18&gt;$B$5),"",D18/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9169,7 +9169,7 @@
         <v/>
       </c>
       <c r="H19" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C19&gt;$B$5),"",D19/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C19&gt;$B$5),"",D19/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9203,7 +9203,7 @@
         <v/>
       </c>
       <c r="H20" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C20&gt;$B$5),"",D20/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C20&gt;$B$5),"",D20/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9237,7 +9237,7 @@
         <v/>
       </c>
       <c r="H21" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C21&gt;$B$5),"",D21/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C21&gt;$B$5),"",D21/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>
@@ -9271,7 +9271,7 @@
         <v/>
       </c>
       <c r="H22" s="20">
-        <f>IF(OR(Parametres!$C$96&lt;=0,C22&gt;$B$5),"",D22/Parametres!$C$96)</f>
+        <f>IF(OR(Parametres!$C$64&lt;=0,C22&gt;$B$5),"",D22/Parametres!$C$64)</f>
         <v/>
       </c>
     </row>

</xml_diff>